<commit_message>
update the file with new changes
</commit_message>
<xml_diff>
--- a/documentation/Speech_to_Text_JIRA_Backlog_Detailed.xlsx
+++ b/documentation/Speech_to_Text_JIRA_Backlog_Detailed.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="61">
   <si>
     <t>Title</t>
   </si>
@@ -185,6 +185,18 @@
   </si>
   <si>
     <t>Nishant</t>
+  </si>
+  <si>
+    <t>Project Documentation SRS,Jira</t>
+  </si>
+  <si>
+    <t>Feature/document-setup</t>
+  </si>
+  <si>
+    <t>Presentation,final Report</t>
+  </si>
+  <si>
+    <t>feature/report</t>
   </si>
 </sst>
 </file>
@@ -516,9 +528,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
+    <col min="1" max="1" width="9.140625" customWidth="1"/>
     <col min="2" max="2" width="82.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="32.5703125" bestFit="1" customWidth="1"/>
@@ -550,19 +563,19 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>57</v>
       </c>
       <c r="C2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D2" t="s">
         <v>7</v>
       </c>
       <c r="E2" t="s">
-        <v>8</v>
+        <v>58</v>
       </c>
       <c r="F2" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -579,7 +592,7 @@
         <v>7</v>
       </c>
       <c r="E3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F3" t="s">
         <v>9</v>
@@ -590,16 +603,16 @@
         <v>0</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="C4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D4" t="s">
-        <v>49</v>
+        <v>7</v>
       </c>
       <c r="E4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F4" t="s">
         <v>9</v>
@@ -610,16 +623,16 @@
         <v>0</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D5" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F5" t="s">
         <v>9</v>
@@ -630,16 +643,16 @@
         <v>0</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C6">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="E6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F6" t="s">
         <v>9</v>
@@ -650,16 +663,16 @@
         <v>0</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C7">
         <v>8</v>
       </c>
       <c r="D7" t="s">
-        <v>7</v>
+        <v>50</v>
       </c>
       <c r="E7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F7" t="s">
         <v>9</v>
@@ -670,16 +683,16 @@
         <v>0</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C8">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D8" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
       <c r="E8" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F8" t="s">
         <v>9</v>
@@ -690,16 +703,16 @@
         <v>0</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C9">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D9" t="s">
         <v>48</v>
       </c>
       <c r="E9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F9" t="s">
         <v>9</v>
@@ -710,16 +723,16 @@
         <v>0</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C10">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D10" t="s">
         <v>48</v>
       </c>
       <c r="E10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F10" t="s">
         <v>9</v>
@@ -730,16 +743,16 @@
         <v>0</v>
       </c>
       <c r="B11" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C11">
         <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E11" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F11" t="s">
         <v>9</v>
@@ -750,16 +763,16 @@
         <v>0</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C12">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D12" t="s">
         <v>51</v>
       </c>
       <c r="E12" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F12" t="s">
         <v>9</v>
@@ -770,16 +783,16 @@
         <v>0</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C13">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E13" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F13" t="s">
         <v>9</v>
@@ -790,19 +803,19 @@
         <v>0</v>
       </c>
       <c r="B14" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C14">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D14" t="s">
-        <v>7</v>
+        <v>52</v>
       </c>
       <c r="E14" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F14" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -810,7 +823,7 @@
         <v>0</v>
       </c>
       <c r="B15" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C15">
         <v>3</v>
@@ -819,7 +832,7 @@
         <v>7</v>
       </c>
       <c r="E15" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F15" t="s">
         <v>33</v>
@@ -830,19 +843,19 @@
         <v>0</v>
       </c>
       <c r="B16" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C16">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D16" t="s">
-        <v>53</v>
+        <v>7</v>
       </c>
       <c r="E16" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F16" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -850,16 +863,16 @@
         <v>0</v>
       </c>
       <c r="B17" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C17">
         <v>5</v>
       </c>
       <c r="D17" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E17" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F17" t="s">
         <v>9</v>
@@ -870,16 +883,16 @@
         <v>0</v>
       </c>
       <c r="B18" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C18">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D18" t="s">
-        <v>7</v>
+        <v>54</v>
       </c>
       <c r="E18" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F18" t="s">
         <v>9</v>
@@ -890,16 +903,16 @@
         <v>0</v>
       </c>
       <c r="B19" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C19">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D19" t="s">
-        <v>48</v>
+        <v>7</v>
       </c>
       <c r="E19" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F19" t="s">
         <v>9</v>
@@ -910,16 +923,16 @@
         <v>0</v>
       </c>
       <c r="B20" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C20">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D20" t="s">
-        <v>7</v>
+        <v>48</v>
       </c>
       <c r="E20" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F20" t="s">
         <v>9</v>
@@ -930,22 +943,63 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
+        <v>44</v>
+      </c>
+      <c r="C21">
+        <v>13</v>
+      </c>
+      <c r="D21" t="s">
+        <v>7</v>
+      </c>
+      <c r="E21" t="s">
+        <v>45</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" t="s">
+        <v>0</v>
+      </c>
+      <c r="B22" t="s">
         <v>46</v>
       </c>
-      <c r="C21">
+      <c r="C22">
         <v>8</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D22" t="s">
         <v>56</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E22" t="s">
         <v>47</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" t="s">
+        <v>0</v>
+      </c>
+      <c r="B23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C23">
+        <v>3</v>
+      </c>
+      <c r="D23" t="s">
+        <v>49</v>
+      </c>
+      <c r="E23" t="s">
+        <v>60</v>
+      </c>
+      <c r="F23" t="s">
         <v>9</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>